<commit_message>
Redis slot hold (task 2.1)
Holds a settled time for a few minutes while the client chooses a therapist - the window an EXCLUDE constraint cannot cover, because no row exists yet. The assistant has been saying the time was held; now something holds it. Capacity is counted rather than boolean so one hesitating client does not empty an hour. Redis unreachable means no hold and booking proceeds exactly as before (NFR#1). REDIS_HOST overridden in compose for the same reason as DB_HOST.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>

Claude-Session: https://claude.ai/code/session_014MbSsgcBwSDdBpZZWJudpn
</commit_message>
<xml_diff>
--- a/HilotSpa_ThesisTracker.xlsx
+++ b/HilotSpa_ThesisTracker.xlsx
@@ -947,7 +947,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:G159"/>
+  <dimension ref="A1:G160"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="11" customWidth="1" style="22" min="1" max="1"/>
@@ -6598,6 +6598,43 @@
       <c r="G159" s="45" t="inlineStr">
         <is>
           <t>Observed live 2026-09-18. Closes B74. Solved WITHOUT a composition feature: each combo is one Massage row with its own duration and price, so the booking engine, the 30-minute slot grid and priceAtBooking all work unchanged, and the duration is stated rather than derived from two parts. The right call for this project.</t>
+        </is>
+      </c>
+    </row>
+    <row r="160" ht="147" customHeight="1" s="23">
+      <c r="A160" s="43" t="inlineStr">
+        <is>
+          <t>Sprint 0</t>
+        </is>
+      </c>
+      <c r="B160" s="44" t="inlineStr">
+        <is>
+          <t>0.34</t>
+        </is>
+      </c>
+      <c r="C160" s="45" t="inlineStr">
+        <is>
+          <t>Decide whether the admin console gets its own hostname</t>
+        </is>
+      </c>
+      <c r="D160" s="45" t="inlineStr">
+        <is>
+          <t>hilotspa-admin.duckdns.org. Adding it is one entry in SITE_HOST and FRONTEND_ORIGIN - the app and API are unchanged.</t>
+        </is>
+      </c>
+      <c r="E160" s="44" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F160" s="44" t="inlineStr">
+        <is>
+          <t>Liodoq</t>
+        </is>
+      </c>
+      <c r="G160" s="45" t="inlineStr">
+        <is>
+          <t>PARKED by Liodoq 2026-09-18, to revisit after node 2. The caveat to weigh then: a separate hostname is PRESENTATION, not protection. Same bundle, same API, so /admin still resolves on the branch hostname and access is decided by the role in the JWT, not by the name typed. Making it mean something requires Caddy refusing /admin/* on the public host, which is doable but buys little while the API is shared.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
tracker: 2.1 Done (Redis slot hold), add 0.35
</commit_message>
<xml_diff>
--- a/HilotSpa_ThesisTracker.xlsx
+++ b/HilotSpa_ThesisTracker.xlsx
@@ -947,7 +947,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:G160"/>
+  <dimension ref="A1:G161"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="11" customWidth="1" style="22" min="1" max="1"/>
@@ -1560,13 +1560,17 @@
       </c>
       <c r="E20" s="35" t="inlineStr">
         <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F20" s="35" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F20" s="35" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
       <c r="G20" s="36" t="inlineStr">
         <is>
-          <t>SUPERSEDED by 2.37, 2026-08-30. Process Rule #4 needed a guarantee that two transactions cannot award the same therapist or room; that guarantee now lives in Postgres as EXCLUDE USING gist, partial on blocking statuses, half-open ranges. A database constraint is strictly stronger than a Redis lock - it cannot be bypassed by a caller that forgets to take it, and it survives a cache restart. Marked N/A rather than Not Started so the sprint total is not understated at the defence.</t>
+          <t>DONE 2026-09-18 and LIVE IN PRODUCTION - verified with a real hold key on the server. Reopened from N/A after Liodoq pushed back on dropping Redis. Claude's first answer was wrong in scope: it argued against Redis as a lock around the booking WRITE, where the V2 EXCLUDE constraints already make double-booking impossible. The actual gap is BEFORE a row exists - between the assistant settling a time and the client choosing a therapist, where there is nothing to constrain and the assistant has been saying 'na-hold na po' about nothing (AssistantServiceImpl even carries a claimsHold() regex to detect the model saying it). A TTL hold is the right tool and Postgres is the wrong one: ephemeral, high-churn, self-expiring. Sorted set per (branch, hour), expiry in the score, pruned on read - no cleanup job, no KEYS scan. capacityAt() replaced the boolean anyFree() because one hesitating client must not empty an hour at a branch with five therapists. Redis unreachable = no hold and booking proceeds exactly as before, so NFR#1 is preserved.</t>
         </is>
       </c>
     </row>
@@ -6635,6 +6639,43 @@
       <c r="G160" s="45" t="inlineStr">
         <is>
           <t>PARKED by Liodoq 2026-09-18, to revisit after node 2. The caveat to weigh then: a separate hostname is PRESENTATION, not protection. Same bundle, same API, so /admin still resolves on the branch hostname and access is decided by the role in the JWT, not by the name typed. Making it mean something requires Caddy refusing /admin/* on the public host, which is doable but buys little while the API is shared.</t>
+        </is>
+      </c>
+    </row>
+    <row r="161" ht="147" customHeight="1" s="23">
+      <c r="A161" s="43" t="inlineStr">
+        <is>
+          <t>Sprint 0</t>
+        </is>
+      </c>
+      <c r="B161" s="44" t="inlineStr">
+        <is>
+          <t>0.35</t>
+        </is>
+      </c>
+      <c r="C161" s="45" t="inlineStr">
+        <is>
+          <t>REDIS_HOST needed a compose override, like DB_HOST and N8N_WEBHOOK_URL</t>
+        </is>
+      </c>
+      <c r="D161" s="45" t="inlineStr">
+        <is>
+          <t>.env says localhost, which is right for run.ps1 and is the BACKEND ITSELF inside the compose network. Added REDIS_HOST: redis and REDIS_PORT: 6379 to the backend's environment block.</t>
+        </is>
+      </c>
+      <c r="E161" s="44" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F161" s="44" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="G161" s="45" t="inlineStr">
+        <is>
+          <t>Third instance of one pattern on 2026-09-18, and the comment block in compose.yaml already documented the other two. Claude added a variable that needed the same treatment and did not give it. Compounded by SlotHoldService logging every failure at DEBUG - 'degrade silently' turned a misconfiguration invisible: every hold was a refused connection and every signal said healthy. Fixed by warning ONCE at WARN then falling back to DEBUG. This is B60's lesson repeating: a fallback that cannot tell 'not attempted' from 'failed' hides the failures you most need to see.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Tracker: node 2 live (3.10), node identity (3.31), B137/B138; fix task ref in comments
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>

Claude-Session: https://claude.ai/code/session_014MbSsgcBwSDdBpZZWJudpn
</commit_message>
<xml_diff>
--- a/HilotSpa_ThesisTracker.xlsx
+++ b/HilotSpa_ThesisTracker.xlsx
@@ -947,7 +947,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:G161"/>
+  <dimension ref="A1:G163"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="11" customWidth="1" style="22" min="1" max="1"/>
@@ -1933,7 +1933,7 @@
       <c r="F31" s="28" t="n"/>
       <c r="G31" s="45" t="inlineStr">
         <is>
-          <t>Half of it is now enforced, and it is the half that can be. 2026-08-30: a therapist and a room each belong to exactly one branch (schema), and Flyway migration V2 adds EXCLUDE constraints so the database itself refuses an overlapping write. Within a node, single-writer is a mechanism rather than a convention. What remains is the cross-node half - a node refusing to write a resource it does not own - which needs the node registry (3.2) to exist first.</t>
+          <t>Half of it is now enforced, and it is the half that can be. 2026-08-30: a therapist and a room each belong to exactly one branch (schema), and Flyway migration V2 adds EXCLUDE constraints so the database itself refuses an overlapping write. Within a node, single-writer is a mechanism rather than a convention. What remains is the cross-node half - a node refusing to write a resource it does not own - which needs the node registry (3.2) to exist first. | 2026-09-18: advanced by 3.31. The data model already made two nodes unable to write the same row; the CLIENT was still choosing the wrong partition. See B137.</t>
         </is>
       </c>
     </row>
@@ -2125,13 +2125,13 @@
       </c>
       <c r="E37" s="28" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F37" s="28" t="n"/>
       <c r="G37" s="45" t="inlineStr">
         <is>
-          <t>Research locale names only one branch. See Defense Risks R5.</t>
+          <t>Node 2 live 2026-09-18: hilotspa-daraga.duckdns.org on its own EC2 (t3.small, Ubuntu 26.04, 2 GB + 2 GB swap, Elastic IP), restored from a pg_dump of node 1, own JWT_SECRET and DB password, certificate obtained first attempt, Redis hold verified. Nothing was deleted anywhere - node 2 HOLDS both branches and WRITES only Daraga. Traps hit and recorded: the security group's rules went into the OUTBOUND list (SSH timed out AND outbound UDP 53 was blocked, so DNS would have failed next); Docker created the bind-mount source ~/hilotSpa/site as ROOT because it did not exist, so the frontend swap failed on an empty site. Runbook: node2-clone-and-split-RUNBOOK.md.</t>
         </is>
       </c>
     </row>
@@ -6676,6 +6676,80 @@
       <c r="G161" s="45" t="inlineStr">
         <is>
           <t>Third instance of one pattern on 2026-09-18, and the comment block in compose.yaml already documented the other two. Claude added a variable that needed the same treatment and did not give it. Compounded by SlotHoldService logging every failure at DEBUG - 'degrade silently' turned a misconfiguration invisible: every hold was a refused connection and every signal said healthy. Fixed by warning ONCE at WARN then falling back to DEBUG. This is B60's lesson repeating: a fallback that cannot tell 'not attempted' from 'failed' hides the failures you most need to see.</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="43" t="inlineStr">
+        <is>
+          <t>Sprint 3</t>
+        </is>
+      </c>
+      <c r="B162" s="44" t="inlineStr">
+        <is>
+          <t>3.31</t>
+        </is>
+      </c>
+      <c r="C162" s="45" t="inlineStr">
+        <is>
+          <t>Node identity - each node names and writes for its own branch</t>
+        </is>
+      </c>
+      <c r="D162" s="45" t="inlineStr">
+        <is>
+          <t>GET /api/v1/public/node returns nodeId, nodeName, branchId, branchName from NODE_BRANCH_ID. Shared NodeStore on the client. The top bar, landing hero, contact, about and the Appendix C signature sheet all read it instead of a literal string, and the assessment files against it instead of branches[0]. The nightly reminder run is scoped to it.</t>
+        </is>
+      </c>
+      <c r="E162" s="44" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F162" s="44" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="G162" s="45" t="inlineStr">
+        <is>
+          <t>Built and deployed 2026-09-18 after node 2 went up and the Daraga site announced itself as Bulan. Closes B137. The startup line "Node X writes for branch Y" is the whole change, verifiable in one grep. A node that declares no branch keeps the old behaviour exactly - a single-node deployment is legitimate - but says so at WARN, because a silent fallback that cannot distinguish "not configured" from "configured" is the B60/0.35 lesson again.</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="43" t="inlineStr">
+        <is>
+          <t>Sprint 3</t>
+        </is>
+      </c>
+      <c r="B163" s="44" t="inlineStr">
+        <is>
+          <t>3.32</t>
+        </is>
+      </c>
+      <c r="C163" s="45" t="inlineStr">
+        <is>
+          <t>Clamp the MANUAL reminder run to the node's own branch</t>
+        </is>
+      </c>
+      <c r="D163" s="45" t="inlineStr">
+        <is>
+          <t>NotificationController.run() uses scopeOf(branchId), which returns null - every branch - for an ADMIN who selects none. The nightly job is scoped by 3.31; the button is not.</t>
+        </is>
+      </c>
+      <c r="E163" s="44" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F163" s="44" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="G163" s="45" t="inlineStr">
+        <is>
+          <t>Opened 2026-09-18. Node 2 keeps MAIL_HOST BLANK until this lands, or an administrator pressing Run reminders there will re-send what node 1 already sent - notification_log is deliberately not replicated, so node 2 cannot know. Needs a product decision first: should an admin on the Daraga node be ABLE to send Bulan reminders at all? Recommendation is no, on the same partitioning argument.</t>
         </is>
       </c>
     </row>
@@ -6710,7 +6784,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:G139"/>
+  <dimension ref="A1:G141"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="7" customWidth="1" style="22" min="1" max="1"/>
@@ -11783,6 +11857,80 @@
       <c r="G139" s="45" t="inlineStr">
         <is>
           <t>Fixed 2026-09-18. The page only knew about the STAFF token; an ADMIN inside a branch context is equally scoped. Same family as B101.</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="44" t="inlineStr">
+        <is>
+          <t>B137</t>
+        </is>
+      </c>
+      <c r="B140" s="44" t="inlineStr">
+        <is>
+          <t>3.31</t>
+        </is>
+      </c>
+      <c r="C140" s="44" t="inlineStr">
+        <is>
+          <t>frontend - review.ts, app-nav, landing, about, contact, protocol-sheet</t>
+        </is>
+      </c>
+      <c r="D140" s="45" t="inlineStr">
+        <is>
+          <t>A customer has no token and therefore no branch, so the assessment fell back to branches[0] - Bulan, alphabetically. On two nodes that meant a client booking on the DARAGA node filed a BULAN appointment. The branch was also a literal string in six templates, including the Appendix C sheet a practitioner signs.</t>
+        </is>
+      </c>
+      <c r="E140" s="44" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F140" s="44" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="G140" s="45" t="inlineStr">
+        <is>
+          <t>Found 2026-09-18 within an hour of node 2 going live: the Daraga site introduced itself as Bulan. Harmless while one node existed, which is why it survived review. Single-writer-per-partition is the property the whole architecture rests on and a DEFAULT was breaking it at the point of entry - the database could not catch it, because a Bulan appointment written by node 2 is a perfectly valid row. Fixed by 3.31. The signed-sheet instance was the worst: a signed protocol table naming the wrong branch asserts that somebody approved rules for a place they never approved them for.</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="44" t="inlineStr">
+        <is>
+          <t>B138</t>
+        </is>
+      </c>
+      <c r="B141" s="44" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C141" s="44" t="inlineStr">
+        <is>
+          <t>node 1 .env</t>
+        </is>
+      </c>
+      <c r="D141" s="45" t="inlineStr">
+        <is>
+          <t>FRONTEND_ORIGIN appears TWICE. Docker Compose takes the last occurrence, so the node works - but anyone editing the first one, which is where you would look, changes nothing.</t>
+        </is>
+      </c>
+      <c r="E141" s="44" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="F141" s="44" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="G141" s="45" t="inlineStr">
+        <is>
+          <t>Found 2026-09-18 while listing key names for node 2. Left from the multi-origin CORS change earlier the same day: the new value was appended instead of replacing the old. Collapse to one line next time node 1 .env is touched.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Body map: drop the impossible front thoracic spot, name every position (K1)
f-thor sat at the centre of the chest carrying region THORACIC, at the same coordinates as its counterpart on the back. The thoracic spine is posterior - there is none on the front of a person - so anyone tapping their sternum was recorded as mid-back pain, indistinguishable from a correct mark on the back view. That matters now that region is about to drive protocol rules. 30 hotspots becomes 29 (13 front, 16 back). Every position also gains a plain-language descriptor, so the two figures stop reading as the same dots twice: Knee - left - kneecap against Knee - left - behind the knee.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>

Claude-Session: https://claude.ai/code/session_014MbSsgcBwSDdBpZZWJudpn
</commit_message>
<xml_diff>
--- a/HilotSpa_ThesisTracker.xlsx
+++ b/HilotSpa_ThesisTracker.xlsx
@@ -947,7 +947,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:G163"/>
+  <dimension ref="A1:G165"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="11" customWidth="1" style="22" min="1" max="1"/>
@@ -1861,13 +1861,13 @@
       </c>
       <c r="E29" s="28" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F29" s="28" t="n"/>
       <c r="G29" s="45" t="inlineStr">
         <is>
-          <t>NEXT. Node registry: table `node` (node_id, name, base_url, branch_id, last_seen_at, last_watermark, state) and GET /api/v1/sync/hello. Auth is a DEDICATED shared secret, never user JWTs - sharing a JWT signing key across nodes means a compromise of either forges logins on both. This is the stage that makes A1's node cards real: an unreachable peer reads 'unreachable, last seen 14:02' rather than being drawn as offline. See claude/sprint3-sync-design.md.</t>
+          <t>NEXT. Node registry: table `node` (node_id, name, base_url, branch_id, last_seen_at, last_watermark, state) and GET /api/v1/sync/hello. Auth is a DEDICATED shared secret, never user JWTs - sharing a JWT signing key across nodes means a compromise of either forges logins on both. This is the stage that makes A1's node cards real: an unreachable peer reads 'unreachable, last seen 14:02' rather than being drawn as offline. See claude/sprint3-sync-design.md. | Built and deployed 2026-09-19. V9 node table; each node writes its own row and polls each configured peer every 30s. Peers are configured as URLs and IDENTITY IS DISCOVERED - a node id in config too means two places can disagree about a name. /api/v1/sync/** is guarded by SyncTokenFilter with a shared secret that DEFAULTS CLOSED, because both nodes publish 443 to the internet for ACME. Constant-time comparison. First run failed 401 on both sides: the generate command had been run on both nodes, producing two different secrets - diagnosed by comparing sha256 fingerprints without either of us seeing the value.</t>
         </is>
       </c>
     </row>
@@ -1894,13 +1894,13 @@
       </c>
       <c r="E30" s="28" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F30" s="28" t="n"/>
       <c r="G30" s="45" t="inlineStr">
         <is>
-          <t>FR#3</t>
+          <t>FR#3 | Built and deployed 2026-09-19. GET /sync/changes?since= returns only rows this node ORIGINATED; GET /sync/appointments?ids= answers only about ids the caller was already told changed - there is no 'list everything'. Appointments cross; accounts, assessments and pain maps are not in sync_log at all, so the puller could not fetch them if it tried. Native ON CONFLICT (id) DO UPDATE rather than save(): the id is @GeneratedValue, and merge on a row absent from this database would let the generator assign a NEW id - silent unbounded duplication on every pull. ReplicationContext (ThreadLocal) stops an applied change being re-advertised, which would otherwise make the two nodes pass the same row back and forth for ever.</t>
         </is>
       </c>
     </row>
@@ -1927,13 +1927,13 @@
       </c>
       <c r="E31" s="28" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F31" s="28" t="n"/>
       <c r="G31" s="45" t="inlineStr">
         <is>
-          <t>Half of it is now enforced, and it is the half that can be. 2026-08-30: a therapist and a room each belong to exactly one branch (schema), and Flyway migration V2 adds EXCLUDE constraints so the database itself refuses an overlapping write. Within a node, single-writer is a mechanism rather than a convention. What remains is the cross-node half - a node refusing to write a resource it does not own - which needs the node registry (3.2) to exist first. | 2026-09-18: advanced by 3.31. The data model already made two nodes unable to write the same row; the CLIENT was still choosing the wrong partition. See B137.</t>
+          <t>Half of it is now enforced, and it is the half that can be. 2026-08-30: a therapist and a room each belong to exactly one branch (schema), and Flyway migration V2 adds EXCLUDE constraints so the database itself refuses an overlapping write. Within a node, single-writer is a mechanism rather than a convention. What remains is the cross-node half - a node refusing to write a resource it does not own - which needs the node registry (3.2) to exist first. | 2026-09-18: advanced by 3.31. The data model already made two nodes unable to write the same row; the CLIENT was still choosing the wrong partition. See B137. | Done 2026-09-19. Now enforced in three places: the data model (a therapist and a room belong to one branch), createForm (the node decides a customer's branch, not the request body - B139), and the reminder clamp (3.32). The client-side fix alone was insufficient: a cached bundle, a stale tab or curl would have bypassed it.</t>
         </is>
       </c>
     </row>
@@ -4852,7 +4852,7 @@
       </c>
       <c r="E112" s="44" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F112" s="44" t="inlineStr">
@@ -4862,7 +4862,7 @@
       </c>
       <c r="G112" s="45" t="inlineStr">
         <is>
-          <t>~30 min and it is the prerequisite for every hosting route. Also removes a whole class of defence-day failure: one thing to start instead of two.</t>
+          <t>~30 min and it is the prerequisite for every hosting route. Also removes a whole class of defence-day failure: one thing to start instead of two. | Done - Caddy serves the bundle and proxies /api on both nodes.</t>
         </is>
       </c>
     </row>
@@ -4889,7 +4889,7 @@
       </c>
       <c r="E113" s="44" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F113" s="44" t="inlineStr">
@@ -4899,7 +4899,7 @@
       </c>
       <c r="G113" s="45" t="inlineStr">
         <is>
-          <t>Needed for a real URL by either route.</t>
+          <t>Needed for a real URL by either route. | Done - Caddy with automatic Let's Encrypt on both nodes; SITE_HOST comes from the environment, never the tracked Caddyfile.</t>
         </is>
       </c>
     </row>
@@ -4926,7 +4926,7 @@
       </c>
       <c r="E114" s="44" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F114" s="44" t="inlineStr">
@@ -4936,7 +4936,7 @@
       </c>
       <c r="G114" s="45" t="inlineStr">
         <is>
-          <t>The panel has asked for a real URL. NOTE: AWS changed the free tier - accounts after 15 Jul 2025 get $100 credits for 12 months, not 750 free hours, and a Free Plan account auto-closes when they run out.</t>
+          <t>The panel has asked for a real URL. NOTE: AWS changed the free tier - accounts after 15 Jul 2025 get $100 credits for 12 months, not 750 free hours, and a Free Plan account auto-closes when they run out. | Done - two EC2 t3.small in ap-southeast-1, both on the same account.</t>
         </is>
       </c>
     </row>
@@ -6739,17 +6739,91 @@
       </c>
       <c r="E163" s="44" t="inlineStr">
         <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F163" s="44" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="G163" s="45" t="inlineStr">
+        <is>
+          <t>Opened 2026-09-18. Node 2 keeps MAIL_HOST BLANK until this lands, or an administrator pressing Run reminders there will re-send what node 1 already sent - notification_log is deliberately not replicated, so node 2 cannot know. Needs a product decision first: should an admin on the Daraga node be ABLE to send Bulan reminders at all? Recommendation is no, on the same partitioning argument. | Done 2026-09-19. sendScope() clamps both send paths to the branch this node owns; an admin asking for every branch gets a 409 naming which machine to use. Reads are deliberately NOT clamped - the row is already in this database; mailing its client is the thing that leaves the building. A8 states which branch the node sends for before anybody presses anything. MAIL_HOST restored on node 2 once node 1 was clamped first.</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" s="43" t="inlineStr">
+        <is>
+          <t>Sprint 3</t>
+        </is>
+      </c>
+      <c r="B164" s="44" t="inlineStr">
+        <is>
+          <t>3.33</t>
+        </is>
+      </c>
+      <c r="C164" s="45" t="inlineStr">
+        <is>
+          <t>Planned therapist leave, and the bookings it breaks</t>
+        </is>
+      </c>
+      <c r="D164" s="45" t="inlineStr">
+        <is>
+          <t>V10 therapist_leave: a dated, inclusive range entered in advance. Filtered per-day inside availability() and enforced in freeTherapists(), which is the gate the WRITE passes through. Recording leave is never refused because of existing bookings - it answers with the clashing visits by name and time.</t>
+        </is>
+      </c>
+      <c r="E164" s="44" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F164" s="44" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="G164" s="45" t="inlineStr">
+        <is>
+          <t>Built 2026-09-19 at the adviser's question. The system had therapist.status (right-now, today only) and therapist.active (has left, for ever) and nothing in between. Deliberately does NOT auto-cancel: the client still wants the treatment, there is no cancellation email in this system, and swapping the practitioner on a bone-setting appointment is a real change rather than a clerical one. KNOWN WEAKNESS raised by the adviser: the clash list lives on the leave record, so it can be missed. The day-sheet warning that closes that hole is task 3.34.</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="43" t="inlineStr">
+        <is>
+          <t>Sprint 3</t>
+        </is>
+      </c>
+      <c r="B165" s="44" t="inlineStr">
+        <is>
+          <t>3.34</t>
+        </is>
+      </c>
+      <c r="C165" s="45" t="inlineStr">
+        <is>
+          <t>Mark bookings whose therapist is on leave, on the day sheet and queue</t>
+        </is>
+      </c>
+      <c r="D165" s="45" t="inlineStr">
+        <is>
+          <t>Surface the clash where staff already look, rather than only on the leave record.</t>
+        </is>
+      </c>
+      <c r="E165" s="44" t="inlineStr">
+        <is>
           <t>Not Started</t>
         </is>
       </c>
-      <c r="F163" s="44" t="inlineStr">
+      <c r="F165" s="44" t="inlineStr">
         <is>
           <t>Claude</t>
         </is>
       </c>
-      <c r="G163" s="45" t="inlineStr">
-        <is>
-          <t>Opened 2026-09-18. Node 2 keeps MAIL_HOST BLANK until this lands, or an administrator pressing Run reminders there will re-send what node 1 already sent - notification_log is deliberately not replicated, so node 2 cannot know. Needs a product decision first: should an admin on the Daraga node be ABLE to send Bulan reminders at all? Recommendation is no, on the same partitioning argument.</t>
+      <c r="G165" s="45" t="inlineStr">
+        <is>
+          <t>Opened 2026-09-19. This is what makes 3.33 defensible: flag-and-decide only works if somebody looks. Enter leave for three weeks ahead, nobody reopens that screen, and the client turns up to a therapist who is not there. ~45 minutes and it does not touch the availability path.</t>
         </is>
       </c>
     </row>
@@ -6784,7 +6858,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:G141"/>
+  <dimension ref="A1:G145"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="7" customWidth="1" style="22" min="1" max="1"/>
@@ -11931,6 +12005,154 @@
       <c r="G141" s="45" t="inlineStr">
         <is>
           <t>Found 2026-09-18 while listing key names for node 2. Left from the multi-origin CORS change earlier the same day: the new value was appended instead of replacing the old. Collapse to one line next time node 1 .env is touched.</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>B139</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>3.31</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>FormsServiceImpl.createForm</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>For a CUSTOMER, branchId was taken straight from the request body. A booking made on the Bulan site was filed against Daraga, because a frontend predating 3.31 falls back to branches[0] and the branch list comes back UNORDERED from the API.</t>
+        </is>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F142" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="G142" t="inlineStr">
+        <is>
+          <t>Found 2026-09-19 by clicking through, not by reading code. The frontend fix shipped the night before was necessary and insufficient - single-writer-per-partition cannot depend on every client being current. Enforced at the writer now. Appointments inherit the form branch, so one change covers availability, the hold, the booking and the reminder. Trap worth remembering: on node 1 the OLD hardcoded "Bulan, Sorsogon" and the correct dynamic value are identical, so the screen Claude checked was the one screen that could not reveal the fault.</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>B140</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>pages/home - customer landing</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>A visit on 20 Sep appears under BOTH "Your next visit" and "Past sessions" while it is still in the future.</t>
+        </is>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="F143" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="G143" t="inlineStr">
+        <is>
+          <t>Found 2026-09-19. Visible on the first screen a client sees, and on a screen the adviser will open.</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>B141</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>deploy-frontend.ps1</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>The swap deletes every file before copying the new build, so any browser tab open at that moment breaks with "Failed to fetch dynamically imported module: chunk-XXXX.js" the next time it navigates.</t>
+        </is>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>Major</t>
+        </is>
+      </c>
+      <c r="F144" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="G144" t="inlineStr">
+        <is>
+          <t>Hit repeatedly on 2026-09-19. Angular lazy chunks carry hashed names; a page holding the old index.html asks for chunks that no longer exist. Fix is to overlay the new build instead of deleting first, and prune old files later. Until then: hard refresh after every deploy, and DO NOT deploy while the adviser has the site open.</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>B142</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>3.32</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>.env on both nodes - MAIL_USERNAME</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>MAIL_USERNAME, MAIL_FROM and MAIL_REPLY_TO carried one extra "s" (kneadwellnesssspa@). Gmail rejected a username that does not exist, which is indistinguishable from a bad password on the admin screen.</t>
+        </is>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>Major</t>
+        </is>
+      </c>
+      <c r="F145" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="G145" t="inlineStr">
+        <is>
+          <t>Fixed 2026-09-19 after a long chase. Earlier causes in the same chain: MAIL_HOST set to the literal placeholder "&lt;the value from node 1&gt;" (Claude's fault for writing a pasteable placeholder - second time, after &lt;paste-a-key-here&gt; in Session 16), and a 19-character MAIL_PASSWORD. Settled only by talking to smtp.gmail.com directly with python3 and reading Google's own words instead of Spring's wrapper. LESSON: when an error message is generic, stop inferring and ask the system that is refusing.</t>
         </is>
       </c>
     </row>

</xml_diff>